<commit_message>
update:  Aira task1 bounty
</commit_message>
<xml_diff>
--- a/reward/task1_bounty.xlsx
+++ b/reward/task1_bounty.xlsx
@@ -10,7 +10,7 @@
     <sheet name="learn_task_submission_report" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">learn_task_submission_report!$A$1:$H$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">learn_task_submission_report!$A$1:$I$53</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="190">
   <si>
     <t>folder</t>
   </si>
@@ -122,10 +122,16 @@
     <t>Aira</t>
   </si>
   <si>
+    <t>aleo1cyd0g6z8xp2vry0kq5tne2sek5c0vmqzuptx023vjz6we9lrxuzqf354rm</t>
+  </si>
+  <si>
+    <t>https://explorer.provable.com/transaction/at14ggar0qncz7kjttaawc968u04h5dlve4ga905q9gy53fq0egg5gs7mdmtn?utm_source=shield</t>
+  </si>
+  <si>
+    <t>Asher-Tan</t>
+  </si>
+  <si>
     <t>未填写</t>
-  </si>
-  <si>
-    <t>Asher-Tan</t>
   </si>
   <si>
     <t>aleo1veez9g7f6n2de55cxggtcq475sdfsf0dx2xwcf7rgxm3ze6stuyskl863w</t>
@@ -1209,11 +1215,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1268,7 +1277,17 @@
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="19">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1472,25 +1491,25 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="7"/>
-      <tableStyleElement type="headerRow" dxfId="6"/>
-      <tableStyleElement type="totalRow" dxfId="5"/>
-      <tableStyleElement type="firstColumn" dxfId="4"/>
-      <tableStyleElement type="lastColumn" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
+      <tableStyleElement type="totalRow" dxfId="6"/>
+      <tableStyleElement type="firstColumn" dxfId="5"/>
+      <tableStyleElement type="lastColumn" dxfId="4"/>
+      <tableStyleElement type="firstRowStripe" dxfId="3"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="2"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="17"/>
-      <tableStyleElement type="totalRow" dxfId="16"/>
-      <tableStyleElement type="firstRowStripe" dxfId="15"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="14"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="13"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="11"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="10"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="9"/>
-      <tableStyleElement type="pageFieldValues" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="18"/>
+      <tableStyleElement type="totalRow" dxfId="17"/>
+      <tableStyleElement type="firstRowStripe" dxfId="16"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="15"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="14"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="13"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="12"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="11"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="10"/>
+      <tableStyleElement type="pageFieldValues" dxfId="9"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1758,7 +1777,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I53"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <cols>
@@ -1944,7 +1963,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -1969,10 +1988,13 @@
       <c r="H7" t="s">
         <v>30</v>
       </c>
+      <c r="I7" s="2" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
         <v>10</v>
@@ -1987,21 +2009,21 @@
         <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
@@ -2016,21 +2038,21 @@
         <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" hidden="1" spans="1:8">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
@@ -2045,18 +2067,18 @@
         <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H10" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" hidden="1" spans="1:8">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
@@ -2071,18 +2093,18 @@
         <v>11</v>
       </c>
       <c r="F11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
@@ -2097,21 +2119,21 @@
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H12" t="s">
         <v>13</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B13" t="s">
         <v>10</v>
@@ -2126,21 +2148,21 @@
         <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" hidden="1" spans="1:8">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
@@ -2155,18 +2177,18 @@
         <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H14" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s">
         <v>10</v>
@@ -2181,21 +2203,21 @@
         <v>11</v>
       </c>
       <c r="F15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
@@ -2210,21 +2232,21 @@
         <v>11</v>
       </c>
       <c r="F16" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
         <v>10</v>
@@ -2239,21 +2261,21 @@
         <v>11</v>
       </c>
       <c r="F17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G17" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H17" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B18" t="s">
         <v>10</v>
@@ -2268,21 +2290,21 @@
         <v>11</v>
       </c>
       <c r="F18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G18" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H18" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B19" t="s">
         <v>10</v>
@@ -2297,21 +2319,21 @@
         <v>11</v>
       </c>
       <c r="F19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" hidden="1" spans="1:9">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B20" t="s">
         <v>11</v>
@@ -2326,21 +2348,21 @@
         <v>11</v>
       </c>
       <c r="F20" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G20" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B21" t="s">
         <v>10</v>
@@ -2355,21 +2377,21 @@
         <v>11</v>
       </c>
       <c r="F21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G21" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H21" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B22" t="s">
         <v>10</v>
@@ -2384,21 +2406,21 @@
         <v>11</v>
       </c>
       <c r="F22" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H22" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B23" t="s">
         <v>10</v>
@@ -2413,21 +2435,21 @@
         <v>11</v>
       </c>
       <c r="F23" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G23" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H23" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B24" t="s">
         <v>10</v>
@@ -2442,21 +2464,21 @@
         <v>11</v>
       </c>
       <c r="F24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H24" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B25" t="s">
         <v>10</v>
@@ -2471,21 +2493,21 @@
         <v>11</v>
       </c>
       <c r="F25" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G25" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H25" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B26" t="s">
         <v>10</v>
@@ -2500,18 +2522,18 @@
         <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G26" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H26" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B27" t="s">
         <v>10</v>
@@ -2526,21 +2548,21 @@
         <v>11</v>
       </c>
       <c r="F27" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B28" t="s">
         <v>10</v>
@@ -2555,18 +2577,18 @@
         <v>11</v>
       </c>
       <c r="F28" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G28" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H28" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B29" t="s">
         <v>10</v>
@@ -2581,21 +2603,21 @@
         <v>11</v>
       </c>
       <c r="F29" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G29" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H29" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B30" t="s">
         <v>10</v>
@@ -2610,21 +2632,21 @@
         <v>11</v>
       </c>
       <c r="F30" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G30" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H30" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B31" t="s">
         <v>10</v>
@@ -2639,21 +2661,21 @@
         <v>11</v>
       </c>
       <c r="F31" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G31" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H31" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="32" hidden="1" spans="1:8">
       <c r="A32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B32" t="s">
         <v>11</v>
@@ -2668,18 +2690,18 @@
         <v>11</v>
       </c>
       <c r="F32" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H32" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:9">
       <c r="A33" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B33" t="s">
         <v>10</v>
@@ -2694,21 +2716,21 @@
         <v>11</v>
       </c>
       <c r="F33" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G33" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H33" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="34" hidden="1" spans="1:8">
       <c r="A34" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B34" t="s">
         <v>11</v>
@@ -2723,18 +2745,18 @@
         <v>11</v>
       </c>
       <c r="F34" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G34" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H34" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:9">
       <c r="A35" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B35" t="s">
         <v>10</v>
@@ -2749,21 +2771,21 @@
         <v>11</v>
       </c>
       <c r="F35" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G35" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H35" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="36" spans="1:9">
       <c r="A36" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B36" t="s">
         <v>10</v>
@@ -2778,21 +2800,21 @@
         <v>11</v>
       </c>
       <c r="F36" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G36" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H36" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:9">
       <c r="A37" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B37" t="s">
         <v>10</v>
@@ -2807,21 +2829,21 @@
         <v>11</v>
       </c>
       <c r="F37" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G37" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H37" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="38" spans="1:9">
       <c r="A38" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B38" t="s">
         <v>10</v>
@@ -2836,21 +2858,21 @@
         <v>11</v>
       </c>
       <c r="F38" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H38" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="39" hidden="1" spans="1:8">
       <c r="A39" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B39" t="s">
         <v>11</v>
@@ -2865,18 +2887,18 @@
         <v>11</v>
       </c>
       <c r="F39" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G39" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H39" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B40" t="s">
         <v>10</v>
@@ -2891,21 +2913,21 @@
         <v>11</v>
       </c>
       <c r="F40" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G40" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H40" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="41" hidden="1" spans="1:8">
       <c r="A41" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B41" t="s">
         <v>11</v>
@@ -2920,18 +2942,18 @@
         <v>11</v>
       </c>
       <c r="F41" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G41" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H41" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="A42" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B42" t="s">
         <v>10</v>
@@ -2946,21 +2968,21 @@
         <v>11</v>
       </c>
       <c r="F42" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G42" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H42" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B43" t="s">
         <v>10</v>
@@ -2975,21 +2997,21 @@
         <v>11</v>
       </c>
       <c r="F43" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G43" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H43" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B44" t="s">
         <v>10</v>
@@ -3004,18 +3026,18 @@
         <v>11</v>
       </c>
       <c r="F44" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="G44" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H44" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="45" hidden="1" spans="1:8">
       <c r="A45" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B45" t="s">
         <v>11</v>
@@ -3030,18 +3052,18 @@
         <v>11</v>
       </c>
       <c r="F45" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G45" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H45" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B46" t="s">
         <v>10</v>
@@ -3056,21 +3078,21 @@
         <v>11</v>
       </c>
       <c r="F46" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G46" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H46" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B47" t="s">
         <v>10</v>
@@ -3085,21 +3107,21 @@
         <v>11</v>
       </c>
       <c r="F47" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G47" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H47" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B48" t="s">
         <v>10</v>
@@ -3114,21 +3136,21 @@
         <v>11</v>
       </c>
       <c r="F48" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G48" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H48" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="49" spans="1:9">
       <c r="A49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B49" t="s">
         <v>10</v>
@@ -3143,21 +3165,21 @@
         <v>11</v>
       </c>
       <c r="F49" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H49" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="50" spans="1:9">
       <c r="A50" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B50" t="s">
         <v>10</v>
@@ -3172,21 +3194,21 @@
         <v>11</v>
       </c>
       <c r="F50" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G50" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H50" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B51" t="s">
         <v>10</v>
@@ -3201,18 +3223,18 @@
         <v>10</v>
       </c>
       <c r="F51" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G51" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="H51" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="52" hidden="1" spans="1:8">
       <c r="A52" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B52" t="s">
         <v>11</v>
@@ -3227,18 +3249,18 @@
         <v>11</v>
       </c>
       <c r="F52" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G52" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="H52" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B53" t="s">
         <v>10</v>
@@ -3253,18 +3275,29 @@
         <v>11</v>
       </c>
       <c r="F53" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G53" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H53" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:I53" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Y"/>
+      </filters>
+    </filterColumn>
+    <extLst/>
+  </autoFilter>
   <conditionalFormatting sqref="G$1:G$1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H$1:H$1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" display="https://explorer.provable.com/transaction/at1jsf2lawu9cfeq4lxtq2jnfaajg2qlf3952w35p87kedhjh58nsgq3wmqfm?utm_source=shield"/>
@@ -3304,6 +3337,7 @@
     <hyperlink ref="I49" r:id="rId35" display="https://explorer.provable.com/transaction/at1ks5sqkwv8pcwl38466lu9fdetwnm086uhhurlapcjvlw7ppcxu9sknjytd?utm_source=shield"/>
     <hyperlink ref="I50" r:id="rId36" display="https://explorer.provable.com/transaction/at1jne56rhc5jfl6k8pq0m8n4kf8042n5ydmh25vjw0vv2mxrmtsyrsnwewey?utm_source=shield"/>
     <hyperlink ref="I20" r:id="rId37" display="https://explorer.provable.com/transaction/at128yalhwr35z4eytfatle9dkfw4040ep7hlld8hly3zv7mkvpnczs0arefv?utm_source=shield" tooltip="https://explorer.provable.com/transaction/at128yalhwr35z4eytfatle9dkfw4040ep7hlld8hly3zv7mkvpnczs0arefv?utm_source=shield"/>
+    <hyperlink ref="I7" r:id="rId38" display="https://explorer.provable.com/transaction/at14ggar0qncz7kjttaawc968u04h5dlve4ga905q9gy53fq0egg5gs7mdmtn?utm_source=shield" tooltip="https://explorer.provable.com/transaction/at14ggar0qncz7kjttaawc968u04h5dlve4ga905q9gy53fq0egg5gs7mdmtn?utm_source=shield"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>